<commit_message>
Update tests to ensure on-par queries
</commit_message>
<xml_diff>
--- a/exports/performance_run_1000.xlsx
+++ b/exports/performance_run_1000.xlsx
@@ -485,19 +485,19 @@
         <v>30</v>
       </c>
       <c r="D2" t="n">
-        <v>0.079</v>
+        <v>0.025</v>
       </c>
       <c r="E2" t="n">
-        <v>0.116</v>
+        <v>0.026</v>
       </c>
       <c r="F2" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.026</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>1170</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="3">
@@ -518,16 +518,16 @@
         <v>0.042</v>
       </c>
       <c r="E3" t="n">
-        <v>0.045</v>
+        <v>0.09</v>
       </c>
       <c r="F3" t="n">
-        <v>0.045</v>
+        <v>0.051</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>1170</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="4">
@@ -545,13 +545,13 @@
         <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="E4" t="n">
         <v>0.008</v>
       </c>
       <c r="F4" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -575,13 +575,13 @@
         <v>30</v>
       </c>
       <c r="D5" t="n">
-        <v>0.476</v>
+        <v>0.454</v>
       </c>
       <c r="E5" t="n">
-        <v>0.502</v>
+        <v>0.574</v>
       </c>
       <c r="F5" t="n">
-        <v>0.472</v>
+        <v>0.469</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -605,19 +605,19 @@
         <v>30</v>
       </c>
       <c r="D6" t="n">
-        <v>0.062</v>
+        <v>0.056</v>
       </c>
       <c r="E6" t="n">
-        <v>0.09</v>
+        <v>0.082</v>
       </c>
       <c r="F6" t="n">
-        <v>0.066</v>
+        <v>0.06</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>1980</v>
+        <v>2070</v>
       </c>
     </row>
     <row r="7">
@@ -635,13 +635,13 @@
         <v>30</v>
       </c>
       <c r="D7" t="n">
-        <v>0.217</v>
+        <v>0.211</v>
       </c>
       <c r="E7" t="n">
-        <v>0.267</v>
+        <v>0.238</v>
       </c>
       <c r="F7" t="n">
-        <v>0.228</v>
+        <v>0.216</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -665,13 +665,13 @@
         <v>30</v>
       </c>
       <c r="D8" t="n">
-        <v>0.599</v>
+        <v>0.618</v>
       </c>
       <c r="E8" t="n">
-        <v>0.665</v>
+        <v>0.636</v>
       </c>
       <c r="F8" t="n">
-        <v>0.599</v>
+        <v>0.611</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -695,13 +695,13 @@
         <v>30</v>
       </c>
       <c r="D9" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
       <c r="E9" t="n">
-        <v>0.061</v>
+        <v>0.047</v>
       </c>
       <c r="F9" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -725,13 +725,13 @@
         <v>30</v>
       </c>
       <c r="D10" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="E10" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="F10" t="n">
         <v>0.026</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.025</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -755,19 +755,19 @@
         <v>30</v>
       </c>
       <c r="D11" t="n">
-        <v>0.29</v>
+        <v>0.431</v>
       </c>
       <c r="E11" t="n">
-        <v>0.332</v>
+        <v>0.502</v>
       </c>
       <c r="F11" t="n">
-        <v>0.305</v>
+        <v>0.438</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>5070</v>
+        <v>5010</v>
       </c>
     </row>
     <row r="12">
@@ -785,13 +785,13 @@
         <v>30</v>
       </c>
       <c r="D12" t="n">
-        <v>0.309</v>
+        <v>0.263</v>
       </c>
       <c r="E12" t="n">
-        <v>0.336</v>
+        <v>0.296</v>
       </c>
       <c r="F12" t="n">
-        <v>0.316</v>
+        <v>0.271</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -815,13 +815,13 @@
         <v>30</v>
       </c>
       <c r="D13" t="n">
-        <v>0.271</v>
+        <v>0.259</v>
       </c>
       <c r="E13" t="n">
-        <v>0.325</v>
+        <v>0.331</v>
       </c>
       <c r="F13" t="n">
-        <v>0.284</v>
+        <v>0.274</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -845,13 +845,13 @@
         <v>30</v>
       </c>
       <c r="D14" t="n">
-        <v>0.216</v>
+        <v>0.207</v>
       </c>
       <c r="E14" t="n">
-        <v>0.245</v>
+        <v>0.262</v>
       </c>
       <c r="F14" t="n">
-        <v>0.227</v>
+        <v>0.219</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -875,13 +875,13 @@
         <v>30</v>
       </c>
       <c r="D15" t="n">
-        <v>0.772</v>
+        <v>0.749</v>
       </c>
       <c r="E15" t="n">
-        <v>0.844</v>
+        <v>0.833</v>
       </c>
       <c r="F15" t="n">
-        <v>0.776</v>
+        <v>0.754</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -905,13 +905,13 @@
         <v>30</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>0.73</v>
+        <v>0.706</v>
       </c>
       <c r="F16" t="n">
-        <v>0.699</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -935,13 +935,13 @@
         <v>30</v>
       </c>
       <c r="D17" t="n">
-        <v>0.398</v>
+        <v>0.364</v>
       </c>
       <c r="E17" t="n">
-        <v>0.476</v>
+        <v>0.393</v>
       </c>
       <c r="F17" t="n">
-        <v>0.405</v>
+        <v>0.374</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -965,13 +965,13 @@
         <v>30</v>
       </c>
       <c r="D18" t="n">
-        <v>0.574</v>
+        <v>0.606</v>
       </c>
       <c r="E18" t="n">
-        <v>0.628</v>
+        <v>0.627</v>
       </c>
       <c r="F18" t="n">
-        <v>0.573</v>
+        <v>0.6</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -995,13 +995,13 @@
         <v>30</v>
       </c>
       <c r="D19" t="n">
-        <v>0.268</v>
+        <v>0.253</v>
       </c>
       <c r="E19" t="n">
-        <v>0.318</v>
+        <v>0.331</v>
       </c>
       <c r="F19" t="n">
-        <v>0.282</v>
+        <v>0.271</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1025,13 +1025,13 @@
         <v>30</v>
       </c>
       <c r="D20" t="n">
-        <v>0.282</v>
+        <v>0.269</v>
       </c>
       <c r="E20" t="n">
-        <v>0.376</v>
+        <v>0.303</v>
       </c>
       <c r="F20" t="n">
-        <v>0.3</v>
+        <v>0.277</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1055,13 +1055,13 @@
         <v>30</v>
       </c>
       <c r="D21" t="n">
-        <v>0.515</v>
+        <v>0.499</v>
       </c>
       <c r="E21" t="n">
-        <v>0.582</v>
+        <v>0.634</v>
       </c>
       <c r="F21" t="n">
-        <v>0.516</v>
+        <v>0.514</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1088,16 +1088,16 @@
         <v>0.04</v>
       </c>
       <c r="E22" t="n">
-        <v>0.049</v>
+        <v>0.065</v>
       </c>
       <c r="F22" t="n">
-        <v>0.043</v>
+        <v>0.048</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1170</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="23">
@@ -1118,16 +1118,16 @@
         <v>0.034</v>
       </c>
       <c r="E23" t="n">
-        <v>0.041</v>
+        <v>0.036</v>
       </c>
       <c r="F23" t="n">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1170</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="24">
@@ -1148,10 +1148,10 @@
         <v>0.007</v>
       </c>
       <c r="E24" t="n">
-        <v>0.012</v>
+        <v>0.008</v>
       </c>
       <c r="F24" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -1175,13 +1175,13 @@
         <v>30</v>
       </c>
       <c r="D25" t="n">
-        <v>0.606</v>
+        <v>0.621</v>
       </c>
       <c r="E25" t="n">
-        <v>0.638</v>
+        <v>0.707</v>
       </c>
       <c r="F25" t="n">
-        <v>0.603</v>
+        <v>0.624</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1205,19 +1205,19 @@
         <v>30</v>
       </c>
       <c r="D26" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="E26" t="n">
         <v>0.04</v>
       </c>
-      <c r="E26" t="n">
-        <v>0.06</v>
-      </c>
       <c r="F26" t="n">
-        <v>0.043</v>
+        <v>0.039</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1380</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="27">
@@ -1235,13 +1235,13 @@
         <v>30</v>
       </c>
       <c r="D27" t="n">
-        <v>0.284</v>
+        <v>0.279</v>
       </c>
       <c r="E27" t="n">
-        <v>0.338</v>
+        <v>0.307</v>
       </c>
       <c r="F27" t="n">
-        <v>0.298</v>
+        <v>0.287</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -1265,13 +1265,13 @@
         <v>30</v>
       </c>
       <c r="D28" t="n">
-        <v>0.298</v>
+        <v>0.385</v>
       </c>
       <c r="E28" t="n">
-        <v>0.326</v>
+        <v>0.447</v>
       </c>
       <c r="F28" t="n">
-        <v>0.306</v>
+        <v>0.4</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>30</v>
       </c>
       <c r="D29" t="n">
-        <v>0.033</v>
+        <v>0.035</v>
       </c>
       <c r="E29" t="n">
-        <v>0.034</v>
+        <v>0.04</v>
       </c>
       <c r="F29" t="n">
-        <v>0.033</v>
+        <v>0.036</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1325,13 +1325,13 @@
         <v>30</v>
       </c>
       <c r="D30" t="n">
-        <v>0.033</v>
+        <v>0.037</v>
       </c>
       <c r="E30" t="n">
-        <v>0.035</v>
+        <v>0.039</v>
       </c>
       <c r="F30" t="n">
-        <v>0.034</v>
+        <v>0.038</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1355,13 +1355,13 @@
         <v>30</v>
       </c>
       <c r="D31" t="n">
-        <v>0.226</v>
+        <v>0.228</v>
       </c>
       <c r="E31" t="n">
-        <v>0.254</v>
+        <v>0.271</v>
       </c>
       <c r="F31" t="n">
-        <v>0.231</v>
+        <v>0.241</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
@@ -1385,13 +1385,13 @@
         <v>30</v>
       </c>
       <c r="D32" t="n">
-        <v>0.113</v>
+        <v>0.108</v>
       </c>
       <c r="E32" t="n">
-        <v>0.14</v>
+        <v>0.156</v>
       </c>
       <c r="F32" t="n">
-        <v>0.117</v>
+        <v>0.119</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -1415,13 +1415,13 @@
         <v>30</v>
       </c>
       <c r="D33" t="n">
-        <v>0.216</v>
+        <v>0.207</v>
       </c>
       <c r="E33" t="n">
-        <v>0.249</v>
+        <v>0.239</v>
       </c>
       <c r="F33" t="n">
-        <v>0.226</v>
+        <v>0.219</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -1445,13 +1445,13 @@
         <v>30</v>
       </c>
       <c r="D34" t="n">
-        <v>0.109</v>
+        <v>0.104</v>
       </c>
       <c r="E34" t="n">
-        <v>0.17</v>
+        <v>0.118</v>
       </c>
       <c r="F34" t="n">
-        <v>0.118</v>
+        <v>0.108</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1475,13 +1475,13 @@
         <v>30</v>
       </c>
       <c r="D35" t="n">
-        <v>0.619</v>
+        <v>0.669</v>
       </c>
       <c r="E35" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="F35" t="n">
-        <v>0.625</v>
+        <v>0.67</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1505,13 +1505,13 @@
         <v>30</v>
       </c>
       <c r="D36" t="n">
-        <v>0.124</v>
+        <v>0.122</v>
       </c>
       <c r="E36" t="n">
-        <v>0.164</v>
+        <v>0.152</v>
       </c>
       <c r="F36" t="n">
-        <v>0.131</v>
+        <v>0.128</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -1535,13 +1535,13 @@
         <v>30</v>
       </c>
       <c r="D37" t="n">
-        <v>0.295</v>
+        <v>0.289</v>
       </c>
       <c r="E37" t="n">
-        <v>0.326</v>
+        <v>0.32</v>
       </c>
       <c r="F37" t="n">
-        <v>0.305</v>
+        <v>0.298</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -1565,13 +1565,13 @@
         <v>30</v>
       </c>
       <c r="D38" t="n">
-        <v>0.316</v>
+        <v>0.404</v>
       </c>
       <c r="E38" t="n">
-        <v>0.354</v>
+        <v>0.43</v>
       </c>
       <c r="F38" t="n">
-        <v>0.325</v>
+        <v>0.409</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -1595,13 +1595,13 @@
         <v>30</v>
       </c>
       <c r="D39" t="n">
-        <v>0.195</v>
+        <v>0.188</v>
       </c>
       <c r="E39" t="n">
-        <v>0.222</v>
+        <v>0.225</v>
       </c>
       <c r="F39" t="n">
-        <v>0.201</v>
+        <v>0.199</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -1625,13 +1625,13 @@
         <v>30</v>
       </c>
       <c r="D40" t="n">
-        <v>0.223</v>
+        <v>0.218</v>
       </c>
       <c r="E40" t="n">
-        <v>0.305</v>
+        <v>0.247</v>
       </c>
       <c r="F40" t="n">
-        <v>0.242</v>
+        <v>0.226</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -1655,13 +1655,13 @@
         <v>30</v>
       </c>
       <c r="D41" t="n">
-        <v>0.236</v>
+        <v>0.237</v>
       </c>
       <c r="E41" t="n">
-        <v>0.286</v>
+        <v>0.301</v>
       </c>
       <c r="F41" t="n">
-        <v>0.249</v>
+        <v>0.25</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
introduce settings for autovacuum
</commit_message>
<xml_diff>
--- a/exports/performance_run_1000.xlsx
+++ b/exports/performance_run_1000.xlsx
@@ -485,13 +485,13 @@
         <v>30</v>
       </c>
       <c r="D2" t="n">
-        <v>0.025</v>
+        <v>0.027</v>
       </c>
       <c r="E2" t="n">
-        <v>0.026</v>
+        <v>0.044</v>
       </c>
       <c r="F2" t="n">
-        <v>0.026</v>
+        <v>0.029</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -515,13 +515,13 @@
         <v>30</v>
       </c>
       <c r="D3" t="n">
-        <v>0.042</v>
+        <v>0.043</v>
       </c>
       <c r="E3" t="n">
-        <v>0.09</v>
+        <v>0.059</v>
       </c>
       <c r="F3" t="n">
-        <v>0.051</v>
+        <v>0.045</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -575,19 +575,19 @@
         <v>30</v>
       </c>
       <c r="D5" t="n">
-        <v>0.454</v>
+        <v>0.237</v>
       </c>
       <c r="E5" t="n">
-        <v>0.574</v>
+        <v>0.284</v>
       </c>
       <c r="F5" t="n">
-        <v>0.469</v>
+        <v>0.248</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>5670</v>
+        <v>5370</v>
       </c>
     </row>
     <row r="6">
@@ -605,19 +605,19 @@
         <v>30</v>
       </c>
       <c r="D6" t="n">
-        <v>0.056</v>
+        <v>0.049</v>
       </c>
       <c r="E6" t="n">
-        <v>0.082</v>
+        <v>0.055</v>
       </c>
       <c r="F6" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>2070</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="7">
@@ -635,19 +635,19 @@
         <v>30</v>
       </c>
       <c r="D7" t="n">
-        <v>0.211</v>
+        <v>0.13</v>
       </c>
       <c r="E7" t="n">
-        <v>0.238</v>
+        <v>0.173</v>
       </c>
       <c r="F7" t="n">
-        <v>0.216</v>
+        <v>0.137</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>3030</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="8">
@@ -665,13 +665,13 @@
         <v>30</v>
       </c>
       <c r="D8" t="n">
-        <v>0.618</v>
+        <v>0.629</v>
       </c>
       <c r="E8" t="n">
-        <v>0.636</v>
+        <v>0.64</v>
       </c>
       <c r="F8" t="n">
-        <v>0.611</v>
+        <v>0.623</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -698,7 +698,7 @@
         <v>0.04</v>
       </c>
       <c r="E9" t="n">
-        <v>0.047</v>
+        <v>0.043</v>
       </c>
       <c r="F9" t="n">
         <v>0.042</v>
@@ -725,13 +725,13 @@
         <v>30</v>
       </c>
       <c r="D10" t="n">
-        <v>0.024</v>
+        <v>0.028</v>
       </c>
       <c r="E10" t="n">
-        <v>0.038</v>
+        <v>0.065</v>
       </c>
       <c r="F10" t="n">
-        <v>0.026</v>
+        <v>0.037</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -755,13 +755,13 @@
         <v>30</v>
       </c>
       <c r="D11" t="n">
-        <v>0.431</v>
+        <v>0.468</v>
       </c>
       <c r="E11" t="n">
-        <v>0.502</v>
+        <v>0.5</v>
       </c>
       <c r="F11" t="n">
-        <v>0.438</v>
+        <v>0.464</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -785,13 +785,13 @@
         <v>30</v>
       </c>
       <c r="D12" t="n">
-        <v>0.263</v>
+        <v>0.334</v>
       </c>
       <c r="E12" t="n">
-        <v>0.296</v>
+        <v>0.386</v>
       </c>
       <c r="F12" t="n">
-        <v>0.271</v>
+        <v>0.335</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -815,13 +815,13 @@
         <v>30</v>
       </c>
       <c r="D13" t="n">
-        <v>0.259</v>
+        <v>0.258</v>
       </c>
       <c r="E13" t="n">
-        <v>0.331</v>
+        <v>0.289</v>
       </c>
       <c r="F13" t="n">
-        <v>0.274</v>
+        <v>0.266</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -845,13 +845,13 @@
         <v>30</v>
       </c>
       <c r="D14" t="n">
-        <v>0.207</v>
+        <v>0.202</v>
       </c>
       <c r="E14" t="n">
-        <v>0.262</v>
+        <v>0.232</v>
       </c>
       <c r="F14" t="n">
-        <v>0.219</v>
+        <v>0.208</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -875,13 +875,13 @@
         <v>30</v>
       </c>
       <c r="D15" t="n">
-        <v>0.749</v>
+        <v>0.829</v>
       </c>
       <c r="E15" t="n">
-        <v>0.833</v>
+        <v>1.111</v>
       </c>
       <c r="F15" t="n">
-        <v>0.754</v>
+        <v>0.864</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -905,13 +905,13 @@
         <v>30</v>
       </c>
       <c r="D16" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.448</v>
       </c>
       <c r="E16" t="n">
-        <v>0.706</v>
+        <v>0.478</v>
       </c>
       <c r="F16" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.459</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -938,10 +938,10 @@
         <v>0.364</v>
       </c>
       <c r="E17" t="n">
-        <v>0.393</v>
+        <v>0.415</v>
       </c>
       <c r="F17" t="n">
-        <v>0.374</v>
+        <v>0.376</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -965,13 +965,13 @@
         <v>30</v>
       </c>
       <c r="D18" t="n">
-        <v>0.606</v>
+        <v>0.62</v>
       </c>
       <c r="E18" t="n">
-        <v>0.627</v>
+        <v>1.086</v>
       </c>
       <c r="F18" t="n">
-        <v>0.6</v>
+        <v>0.727</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -995,13 +995,13 @@
         <v>30</v>
       </c>
       <c r="D19" t="n">
-        <v>0.253</v>
+        <v>0.264</v>
       </c>
       <c r="E19" t="n">
-        <v>0.331</v>
+        <v>0.444</v>
       </c>
       <c r="F19" t="n">
-        <v>0.271</v>
+        <v>0.304</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1025,13 +1025,13 @@
         <v>30</v>
       </c>
       <c r="D20" t="n">
-        <v>0.269</v>
+        <v>0.288</v>
       </c>
       <c r="E20" t="n">
-        <v>0.303</v>
+        <v>0.443</v>
       </c>
       <c r="F20" t="n">
-        <v>0.277</v>
+        <v>0.311</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1055,13 +1055,13 @@
         <v>30</v>
       </c>
       <c r="D21" t="n">
-        <v>0.499</v>
+        <v>0.525</v>
       </c>
       <c r="E21" t="n">
-        <v>0.634</v>
+        <v>0.552</v>
       </c>
       <c r="F21" t="n">
-        <v>0.514</v>
+        <v>0.523</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1085,19 +1085,19 @@
         <v>30</v>
       </c>
       <c r="D22" t="n">
-        <v>0.04</v>
+        <v>0.019</v>
       </c>
       <c r="E22" t="n">
-        <v>0.065</v>
+        <v>0.02</v>
       </c>
       <c r="F22" t="n">
-        <v>0.048</v>
+        <v>0.02</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1200</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23">
@@ -1115,19 +1115,19 @@
         <v>30</v>
       </c>
       <c r="D23" t="n">
-        <v>0.034</v>
+        <v>0.016</v>
       </c>
       <c r="E23" t="n">
-        <v>0.036</v>
+        <v>0.03</v>
       </c>
       <c r="F23" t="n">
-        <v>0.034</v>
+        <v>0.018</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1200</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24">
@@ -1175,19 +1175,19 @@
         <v>30</v>
       </c>
       <c r="D25" t="n">
-        <v>0.621</v>
+        <v>0.651</v>
       </c>
       <c r="E25" t="n">
-        <v>0.707</v>
+        <v>0.763</v>
       </c>
       <c r="F25" t="n">
-        <v>0.624</v>
+        <v>0.668</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1560</v>
+        <v>240</v>
       </c>
     </row>
     <row r="26">
@@ -1205,19 +1205,19 @@
         <v>30</v>
       </c>
       <c r="D26" t="n">
-        <v>0.038</v>
+        <v>0.018</v>
       </c>
       <c r="E26" t="n">
-        <v>0.04</v>
+        <v>0.044</v>
       </c>
       <c r="F26" t="n">
-        <v>0.039</v>
+        <v>0.022</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1290</v>
+        <v>90</v>
       </c>
     </row>
     <row r="27">
@@ -1235,19 +1235,19 @@
         <v>30</v>
       </c>
       <c r="D27" t="n">
-        <v>0.279</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>0.307</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="F27" t="n">
-        <v>0.287</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1560</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="28">
@@ -1265,13 +1265,13 @@
         <v>30</v>
       </c>
       <c r="D28" t="n">
-        <v>0.385</v>
+        <v>0.399</v>
       </c>
       <c r="E28" t="n">
-        <v>0.447</v>
+        <v>0.477</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4</v>
+        <v>0.414</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1295,19 +1295,19 @@
         <v>30</v>
       </c>
       <c r="D29" t="n">
-        <v>0.035</v>
+        <v>0.016</v>
       </c>
       <c r="E29" t="n">
-        <v>0.04</v>
+        <v>0.018</v>
       </c>
       <c r="F29" t="n">
-        <v>0.036</v>
+        <v>0.017</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1200</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30">
@@ -1325,19 +1325,19 @@
         <v>30</v>
       </c>
       <c r="D30" t="n">
-        <v>0.037</v>
+        <v>0.017</v>
       </c>
       <c r="E30" t="n">
-        <v>0.039</v>
+        <v>0.026</v>
       </c>
       <c r="F30" t="n">
-        <v>0.038</v>
+        <v>0.02</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1200</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31">
@@ -1355,19 +1355,19 @@
         <v>30</v>
       </c>
       <c r="D31" t="n">
-        <v>0.228</v>
+        <v>0.159</v>
       </c>
       <c r="E31" t="n">
-        <v>0.271</v>
+        <v>0.163</v>
       </c>
       <c r="F31" t="n">
-        <v>0.241</v>
+        <v>0.161</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1560</v>
+        <v>300</v>
       </c>
     </row>
     <row r="32">
@@ -1385,13 +1385,13 @@
         <v>30</v>
       </c>
       <c r="D32" t="n">
-        <v>0.108</v>
+        <v>0.112</v>
       </c>
       <c r="E32" t="n">
-        <v>0.156</v>
+        <v>0.135</v>
       </c>
       <c r="F32" t="n">
-        <v>0.119</v>
+        <v>0.115</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -1415,13 +1415,13 @@
         <v>30</v>
       </c>
       <c r="D33" t="n">
-        <v>0.207</v>
+        <v>0.202</v>
       </c>
       <c r="E33" t="n">
-        <v>0.239</v>
+        <v>0.227</v>
       </c>
       <c r="F33" t="n">
-        <v>0.219</v>
+        <v>0.209</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -1445,13 +1445,13 @@
         <v>30</v>
       </c>
       <c r="D34" t="n">
-        <v>0.104</v>
+        <v>0.096</v>
       </c>
       <c r="E34" t="n">
-        <v>0.118</v>
+        <v>0.121</v>
       </c>
       <c r="F34" t="n">
-        <v>0.108</v>
+        <v>0.1</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1475,13 +1475,13 @@
         <v>30</v>
       </c>
       <c r="D35" t="n">
-        <v>0.669</v>
+        <v>0.748</v>
       </c>
       <c r="E35" t="n">
-        <v>0.73</v>
+        <v>0.804</v>
       </c>
       <c r="F35" t="n">
-        <v>0.67</v>
+        <v>0.738</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1505,13 +1505,13 @@
         <v>30</v>
       </c>
       <c r="D36" t="n">
-        <v>0.122</v>
+        <v>0.116</v>
       </c>
       <c r="E36" t="n">
-        <v>0.152</v>
+        <v>0.142</v>
       </c>
       <c r="F36" t="n">
-        <v>0.128</v>
+        <v>0.12</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -1535,13 +1535,13 @@
         <v>30</v>
       </c>
       <c r="D37" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="E37" t="n">
-        <v>0.32</v>
+        <v>0.316</v>
       </c>
       <c r="F37" t="n">
-        <v>0.298</v>
+        <v>0.295</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -1565,13 +1565,13 @@
         <v>30</v>
       </c>
       <c r="D38" t="n">
-        <v>0.404</v>
+        <v>0.411</v>
       </c>
       <c r="E38" t="n">
-        <v>0.43</v>
+        <v>0.549</v>
       </c>
       <c r="F38" t="n">
-        <v>0.409</v>
+        <v>0.433</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -1595,13 +1595,13 @@
         <v>30</v>
       </c>
       <c r="D39" t="n">
-        <v>0.188</v>
+        <v>0.187</v>
       </c>
       <c r="E39" t="n">
-        <v>0.225</v>
+        <v>0.238</v>
       </c>
       <c r="F39" t="n">
-        <v>0.199</v>
+        <v>0.198</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -1625,13 +1625,13 @@
         <v>30</v>
       </c>
       <c r="D40" t="n">
-        <v>0.218</v>
+        <v>0.226</v>
       </c>
       <c r="E40" t="n">
-        <v>0.247</v>
+        <v>0.268</v>
       </c>
       <c r="F40" t="n">
-        <v>0.226</v>
+        <v>0.233</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -1655,13 +1655,13 @@
         <v>30</v>
       </c>
       <c r="D41" t="n">
-        <v>0.237</v>
+        <v>0.245</v>
       </c>
       <c r="E41" t="n">
-        <v>0.301</v>
+        <v>0.273</v>
       </c>
       <c r="F41" t="n">
-        <v>0.25</v>
+        <v>0.253</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>

</xml_diff>